<commit_message>
Trim repetitive supplementary table prose without changing results
</commit_message>
<xml_diff>
--- a/supp/Supplementary_Table_S4_PUBLICATION.xlsx
+++ b/supp/Supplementary_Table_S4_PUBLICATION.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1_GSE210616_patient" sheetId="1" r:id="R9adb7dd51fbe4de5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2_GSE210616_section" sheetId="2" r:id="R30fdc061ff7543b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3_LeeL" sheetId="3" r:id="R635079a612bb4fb7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4_spatial_functional_programs" sheetId="4" r:id="R442e8c71f49b45c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5_paired_sections" sheetId="5" r:id="R4b4325e8d58540e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6_BSW2_patient" sheetId="6" r:id="Re02902ff3e8648d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7_BSW2_provenance" sheetId="7" r:id="Rc8dbc23d373043fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8_sensitivity_LOO" sheetId="8" r:id="Ra4c52b382c9c412a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1_GSE210616_patient" sheetId="1" r:id="R531ba495ffff4ace"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2_GSE210616_section" sheetId="2" r:id="Rb023896b48ad42ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3_LeeL" sheetId="3" r:id="Rbfc55e1d9f4c4d04"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4_spatial_functional_programs" sheetId="4" r:id="R3a263422f6a045f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5_paired_sections" sheetId="5" r:id="Ra220ff519df942c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6_BSW2_patient" sheetId="6" r:id="R5653cff250704827"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7_BSW2_provenance" sheetId="7" r:id="R9809131b9cb547bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8_sensitivity_LOO" sheetId="8" r:id="Rd3329342990744a7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -512,7 +512,7 @@
         <x:v>PATIENT</x:v>
       </x:c>
       <x:c r="N5" s="12" t="str">
-        <x:v>Patient-level spatial association in mixed-cell Visium spots; no malignant-cell-specific or causal claim.</x:v>
+        <x:v>Patient-level association in mixed-cell Visium spots.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -556,7 +556,7 @@
         <x:v>PATIENT</x:v>
       </x:c>
       <x:c r="N6" s="13" t="str">
-        <x:v>Patient-level spatial association in mixed-cell Visium spots; no malignant-cell-specific or causal claim.</x:v>
+        <x:v>Patient-level association in mixed-cell Visium spots.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -600,7 +600,7 @@
         <x:v>PATIENT</x:v>
       </x:c>
       <x:c r="N7" s="12" t="str">
-        <x:v>Patient-level spatial association in mixed-cell Visium spots; no malignant-cell-specific or causal claim.</x:v>
+        <x:v>Patient-level association in mixed-cell Visium spots.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -644,7 +644,7 @@
         <x:v>PATIENT</x:v>
       </x:c>
       <x:c r="N8" s="13" t="str">
-        <x:v>Patient-level spatial association in mixed-cell Visium spots; no malignant-cell-specific or causal claim.</x:v>
+        <x:v>Patient-level association in mixed-cell Visium spots.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -688,7 +688,7 @@
         <x:v>PATIENT</x:v>
       </x:c>
       <x:c r="N9" s="12" t="str">
-        <x:v>Patient-level spatial association in mixed-cell Visium spots; no malignant-cell-specific or causal claim.</x:v>
+        <x:v>Patient-level association in mixed-cell Visium spots.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -732,7 +732,7 @@
         <x:v>PATIENT</x:v>
       </x:c>
       <x:c r="N10" s="13" t="str">
-        <x:v>Patient-level spatial association in mixed-cell Visium spots; no malignant-cell-specific or causal claim.</x:v>
+        <x:v>Patient-level association in mixed-cell Visium spots.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -776,7 +776,7 @@
         <x:v>PATIENT</x:v>
       </x:c>
       <x:c r="N11" s="12" t="str">
-        <x:v>Patient-level spatial association in mixed-cell Visium spots; no malignant-cell-specific or causal claim.</x:v>
+        <x:v>Patient-level association in mixed-cell Visium spots.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -820,7 +820,7 @@
         <x:v>PATIENT</x:v>
       </x:c>
       <x:c r="N12" s="13" t="str">
-        <x:v>Patient-level spatial association in mixed-cell Visium spots; no malignant-cell-specific or causal claim.</x:v>
+        <x:v>Patient-level association in mixed-cell Visium spots.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -864,7 +864,7 @@
         <x:v>PATIENT</x:v>
       </x:c>
       <x:c r="N13" s="12" t="str">
-        <x:v>Patient-level spatial association in mixed-cell Visium spots; no malignant-cell-specific or causal claim.</x:v>
+        <x:v>Patient-level association in mixed-cell Visium spots.</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -908,7 +908,7 @@
         <x:v>PATIENT</x:v>
       </x:c>
       <x:c r="N14" s="13" t="str">
-        <x:v>Patient-level spatial association in mixed-cell Visium spots; no malignant-cell-specific or causal claim.</x:v>
+        <x:v>Patient-level association in mixed-cell Visium spots.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -952,7 +952,7 @@
         <x:v>PATIENT</x:v>
       </x:c>
       <x:c r="N15" s="12" t="str">
-        <x:v>Patient-level spatial association in mixed-cell Visium spots; no malignant-cell-specific or causal claim.</x:v>
+        <x:v>Patient-level association in mixed-cell Visium spots.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -996,7 +996,7 @@
         <x:v>PATIENT</x:v>
       </x:c>
       <x:c r="N16" s="13" t="str">
-        <x:v>Patient-level spatial association in mixed-cell Visium spots; no malignant-cell-specific or causal claim.</x:v>
+        <x:v>Patient-level association in mixed-cell Visium spots.</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -1040,7 +1040,7 @@
         <x:v>PATIENT</x:v>
       </x:c>
       <x:c r="N17" s="12" t="str">
-        <x:v>Patient-level spatial association in mixed-cell Visium spots; no malignant-cell-specific or causal claim.</x:v>
+        <x:v>Patient-level association in mixed-cell Visium spots.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -1084,7 +1084,7 @@
         <x:v>PATIENT</x:v>
       </x:c>
       <x:c r="N18" s="13" t="str">
-        <x:v>Patient-level spatial association in mixed-cell Visium spots; no malignant-cell-specific or causal claim.</x:v>
+        <x:v>Patient-level association in mixed-cell Visium spots.</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -1128,7 +1128,7 @@
         <x:v>PATIENT</x:v>
       </x:c>
       <x:c r="N19" s="12" t="str">
-        <x:v>Patient-level spatial association in mixed-cell Visium spots; no malignant-cell-specific or causal claim.</x:v>
+        <x:v>Patient-level association in mixed-cell Visium spots.</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -1172,7 +1172,7 @@
         <x:v>PATIENT</x:v>
       </x:c>
       <x:c r="N20" s="13" t="str">
-        <x:v>Patient-level spatial association in mixed-cell Visium spots; no malignant-cell-specific or causal claim.</x:v>
+        <x:v>Patient-level association in mixed-cell Visium spots.</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -1216,7 +1216,7 @@
         <x:v>PATIENT</x:v>
       </x:c>
       <x:c r="N21" s="12" t="str">
-        <x:v>Patient-level spatial association in mixed-cell Visium spots; no malignant-cell-specific or causal claim.</x:v>
+        <x:v>Patient-level association in mixed-cell Visium spots.</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -1260,7 +1260,7 @@
         <x:v>PATIENT</x:v>
       </x:c>
       <x:c r="N22" s="13" t="str">
-        <x:v>Patient-level spatial association in mixed-cell Visium spots; no malignant-cell-specific or causal claim.</x:v>
+        <x:v>Patient-level association in mixed-cell Visium spots.</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -1304,7 +1304,7 @@
         <x:v>PATIENT</x:v>
       </x:c>
       <x:c r="N23" s="12" t="str">
-        <x:v>Patient-level spatial association in mixed-cell Visium spots; no malignant-cell-specific or causal claim.</x:v>
+        <x:v>Patient-level association in mixed-cell Visium spots.</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -1348,7 +1348,7 @@
         <x:v>PATIENT</x:v>
       </x:c>
       <x:c r="N24" s="13" t="str">
-        <x:v>Patient-level spatial association in mixed-cell Visium spots; no malignant-cell-specific or causal claim.</x:v>
+        <x:v>Patient-level association in mixed-cell Visium spots.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -1392,7 +1392,7 @@
         <x:v>PATIENT</x:v>
       </x:c>
       <x:c r="N25" s="12" t="str">
-        <x:v>Patient-level spatial association in mixed-cell Visium spots; no malignant-cell-specific or causal claim.</x:v>
+        <x:v>Patient-level association in mixed-cell Visium spots.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -1436,7 +1436,7 @@
         <x:v>PATIENT</x:v>
       </x:c>
       <x:c r="N26" s="13" t="str">
-        <x:v>Patient-level spatial association in mixed-cell Visium spots; no malignant-cell-specific or causal claim.</x:v>
+        <x:v>Patient-level association in mixed-cell Visium spots.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -15403,7 +15403,7 @@
   <x:sheetData>
     <x:row r="1" ht="24" customHeight="1">
       <x:c r="A1" s="2" t="str">
-        <x:v>Supplementary Table S4. BSW2 provenance and implementation assessment</x:v>
+        <x:v>Supplementary Table S4. BSW2 data and methods</x:v>
       </x:c>
       <x:c r="B1" s="2"/>
       <x:c r="C1" s="2"/>

</xml_diff>